<commit_message>
make xlsx to standard layout and add period filters
</commit_message>
<xml_diff>
--- a/api/templates/global_fund_inventory_report/en.xlsx
+++ b/api/templates/global_fund_inventory_report/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\maiki\.oh-my-zsh\aspect\api\templates\global_fund_inventory_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA049939-EA75-4F6D-8FC2-8C99748D39ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A14FC449-9279-4A64-8A7D-1D26043170A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{117EF2D3-2427-48E6-81B8-84AF0A726243}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>#Deployment</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Expiration Date</t>
   </si>
   <si>
-    <t>Stock from last Reporting Month</t>
-  </si>
-  <si>
     <t>Receive during reporting month</t>
   </si>
   <si>
@@ -63,12 +60,6 @@
     <t>Stock at the reporting Time</t>
   </si>
   <si>
-    <t>&lt;Dates&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Table&gt;</t>
-  </si>
-  <si>
     <t>&lt;lotNumber&gt;</t>
   </si>
   <si>
@@ -94,6 +85,24 @@
   </si>
   <si>
     <t>&lt;siteName&gt;</t>
+  </si>
+  <si>
+    <t>Dates: &lt;Dates&gt;</t>
+  </si>
+  <si>
+    <t>States: &lt;States&gt;</t>
+  </si>
+  <si>
+    <t>LGA: &lt;Lgas&gt;</t>
+  </si>
+  <si>
+    <t>&lt;table&gt;</t>
+  </si>
+  <si>
+    <t>Stock from previous period</t>
+  </si>
+  <si>
+    <t>Global Fund Inventory</t>
   </si>
 </sst>
 </file>
@@ -109,8 +118,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -126,7 +135,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -140,16 +149,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -158,18 +167,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0194E0DD-4806-4327-81DB-8345A3306597}">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
@@ -498,97 +501,109 @@
     <col min="9" max="9" width="24.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="1"/>
-      <c r="B1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="E8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s">
+      <c r="G8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E4" t="s">
+      <c r="H8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D15" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1:I1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add report dynamic columns
</commit_message>
<xml_diff>
--- a/api/templates/global_fund_inventory_report/en.xlsx
+++ b/api/templates/global_fund_inventory_report/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\maiki\.oh-my-zsh\aspect\api\templates\global_fund_inventory_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A14FC449-9279-4A64-8A7D-1D26043170A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FD82F56-2542-4F7B-8AD4-AA52AA017501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{117EF2D3-2427-48E6-81B8-84AF0A726243}"/>
   </bookViews>
@@ -34,56 +34,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>#Deployment</t>
   </si>
   <si>
-    <t>Lot Number</t>
-  </si>
-  <si>
-    <t>Expiration Date</t>
-  </si>
-  <si>
-    <t>Receive during reporting month</t>
-  </si>
-  <si>
-    <t>Transfer</t>
-  </si>
-  <si>
-    <t>Use</t>
-  </si>
-  <si>
-    <t>Damage</t>
-  </si>
-  <si>
-    <t>Stock at the reporting Time</t>
-  </si>
-  <si>
-    <t>&lt;lotNumber&gt;</t>
-  </si>
-  <si>
-    <t>&lt;expiresOn&gt;</t>
-  </si>
-  <si>
-    <t>&lt;stockLastMonth&gt;</t>
-  </si>
-  <si>
-    <t>&lt;transferFrom&gt;</t>
-  </si>
-  <si>
-    <t>&lt;receiveTo&gt;</t>
-  </si>
-  <si>
-    <t>&lt;use&gt;</t>
-  </si>
-  <si>
-    <t>&lt;quantityOnHand&gt;</t>
-  </si>
-  <si>
-    <t>&lt;damage&gt;</t>
-  </si>
-  <si>
     <t>&lt;siteName&gt;</t>
   </si>
   <si>
@@ -97,9 +52,6 @@
   </si>
   <si>
     <t>&lt;table&gt;</t>
-  </si>
-  <si>
-    <t>Stock from previous period</t>
   </si>
   <si>
     <t>Global Fund Inventory</t>
@@ -503,22 +455,22 @@
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -534,7 +486,7 @@
     </row>
     <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -549,59 +501,19 @@
       <c r="A7" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>14</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: fix wrokn template tag
</commit_message>
<xml_diff>
--- a/api/templates/global_fund_inventory_report/en.xlsx
+++ b/api/templates/global_fund_inventory_report/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\maiki\.oh-my-zsh\aspect\api\templates\global_fund_inventory_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FD82F56-2542-4F7B-8AD4-AA52AA017501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30CA740E-0BA6-468B-8F06-208688B995D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{117EF2D3-2427-48E6-81B8-84AF0A726243}"/>
   </bookViews>
@@ -51,10 +51,10 @@
     <t>LGA: &lt;Lgas&gt;</t>
   </si>
   <si>
-    <t>&lt;table&gt;</t>
-  </si>
-  <si>
     <t>Global Fund Inventory</t>
+  </si>
+  <si>
+    <t>&lt;Table&gt;</t>
   </si>
 </sst>
 </file>
@@ -455,7 +455,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -486,7 +486,7 @@
     </row>
     <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>

</xml_diff>

<commit_message>
[feat/ASP-2692-Vietnam-Report-M4B3] Addressed report color
</commit_message>
<xml_diff>
--- a/api/templates/global_fund_inventory_report/en.xlsx
+++ b/api/templates/global_fund_inventory_report/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\maiki\.oh-my-zsh\aspect\api\templates\global_fund_inventory_report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\ahernandez\repos\aspect\api\templates\global_fund_inventory_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30CA740E-0BA6-468B-8F06-208688B995D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E033B10-7C8D-40F3-9310-D8597D681F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{117EF2D3-2427-48E6-81B8-84AF0A726243}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117EF2D3-2427-48E6-81B8-84AF0A726243}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -77,6 +77,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -87,8 +93,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FF3CC0DD"/>
       </patternFill>
     </fill>
   </fills>
@@ -124,7 +129,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -143,7 +148,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -440,9 +445,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0194E0DD-4806-4327-81DB-8345A3306597}">
   <dimension ref="A1:I8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.77734375" customWidth="1"/>
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29" bestFit="1" customWidth="1"/>
@@ -479,7 +484,6 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -492,12 +496,11 @@
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>0</v>
       </c>

</xml_diff>